<commit_message>
Checkpoint before single-folder reorg
In-progress work across the app: advanced-config UI rework (simUi),
Lambert/report updates, index.html + styles refresh, new shared-password
auth module (auth.js), and deploy tooling (.htaccess, deploy.sh).

Also makes module cache-busting consistent: every local import now carries
?v=4.6 (incl. the worker URL and the simFlowAlgorithms/ + simConstants chain),
so a version bump invalidates the whole graph and the duplicate simConstants
fetch is gone.

Ignore the regenerable deploy/ build mirror and scratch __queuestorage__.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/Marslink-AI-datacenters.xlsx
+++ b/excel/Marslink-AI-datacenters.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Julien\Documents\git\Space\marslink\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C99FBFA-3992-48EA-ABBB-F3E5DF5D2D0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA2567C3-E28D-4BA5-84D3-FBE206AADBFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="24892" windowHeight="14914" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19107" yWindow="-4060" windowWidth="16186" windowHeight="25787" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AI" sheetId="1" r:id="rId1"/>
@@ -706,6 +706,61 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Sat count</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="#,##0" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -768,6 +823,61 @@
             <a:effectLst/>
           </c:spPr>
         </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Total Mbps</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
         <c:numFmt formatCode="#,##0" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
@@ -1421,16 +1531,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>595993</xdr:colOff>
-      <xdr:row>63</xdr:row>
-      <xdr:rowOff>163285</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>868138</xdr:colOff>
+      <xdr:row>77</xdr:row>
+      <xdr:rowOff>90107</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>639536</xdr:colOff>
-      <xdr:row>76</xdr:row>
-      <xdr:rowOff>141513</xdr:rowOff>
+      <xdr:colOff>260653</xdr:colOff>
+      <xdr:row>96</xdr:row>
+      <xdr:rowOff>182033</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>

</xml_diff>